<commit_message>
Realizo otro ejercicio de ABACUS
</commit_message>
<xml_diff>
--- a/abacus/ejercicio3Abacus.xlsx
+++ b/abacus/ejercicio3Abacus.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ignacio\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ignacio\Desktop\Archivos\VirtualMachine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CD7FDC4-DDC0-4EDD-8BB8-3EA4839F6276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EC7B0E63-57D8-4F72-8ABB-559CEB3421A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="91">
   <si>
     <t>Como pense la solucion:</t>
   </si>
@@ -177,9 +177,6 @@
     <t>Se Carga</t>
   </si>
   <si>
-    <t>Se almacena instrucción carga en 305</t>
-  </si>
-  <si>
     <t>Se genera instrucción carga en acumulador</t>
   </si>
   <si>
@@ -295,6 +292,12 @@
   </si>
   <si>
     <t>Lo sumo con el complemento del contenido del vector o el contenido del vector, depende el caso</t>
+  </si>
+  <si>
+    <t>Se almacena instrucción carga en 309</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   HARDCODEADO. Hay que cargar instrucción 300, sumarle 1 y sumarle desplazamiento</t>
   </si>
 </sst>
 </file>
@@ -454,7 +457,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -587,13 +590,6 @@
     <xf numFmtId="165" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -945,7 +941,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B32:D149"/>
+  <dimension ref="B32:E149"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.140625" customWidth="1"/>
@@ -1012,7 +1008,7 @@
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B43" s="27" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C43" s="27"/>
       <c r="D43" s="27"/>
@@ -1068,7 +1064,7 @@
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B51" s="53" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C51" s="53"/>
       <c r="D51" s="53"/>
@@ -1115,37 +1111,17 @@
     </row>
     <row r="59" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B59" s="32" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C59" s="32"/>
       <c r="D59" s="32"/>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B60" s="61" t="s">
-        <v>85</v>
-      </c>
-      <c r="C60" s="61"/>
-      <c r="D60" s="61"/>
-    </row>
-    <row r="61" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B61" s="58"/>
-      <c r="C61" s="58"/>
-      <c r="D61" s="58"/>
-    </row>
-    <row r="62" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B62" s="58"/>
-      <c r="C62" s="58"/>
-      <c r="D62" s="58"/>
-    </row>
-    <row r="63" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B63" s="58"/>
-      <c r="C63" s="58"/>
-      <c r="D63" s="58"/>
-    </row>
-    <row r="64" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B64" s="58"/>
-      <c r="C64" s="58"/>
-      <c r="D64" s="58"/>
+      <c r="B60" s="58" t="s">
+        <v>84</v>
+      </c>
+      <c r="C60" s="58"/>
+      <c r="D60" s="58"/>
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B75" s="1" t="s">
@@ -1246,7 +1222,7 @@
         <v>26</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="85" spans="2:4" x14ac:dyDescent="0.25">
@@ -1257,7 +1233,7 @@
         <v>0</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="86" spans="2:4" x14ac:dyDescent="0.25">
@@ -1268,7 +1244,7 @@
         <v>3</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="87" spans="2:4" x14ac:dyDescent="0.25">
@@ -1297,7 +1273,7 @@
         <v>1300</v>
       </c>
       <c r="D89" s="15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="90" spans="2:4" x14ac:dyDescent="0.25">
@@ -1308,7 +1284,7 @@
         <v>3255</v>
       </c>
       <c r="D90" s="15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="91" spans="2:4" x14ac:dyDescent="0.25">
@@ -1319,7 +1295,7 @@
         <v>2304</v>
       </c>
       <c r="D91" s="15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="92" spans="2:4" x14ac:dyDescent="0.25">
@@ -1330,7 +1306,7 @@
         <v>26</v>
       </c>
       <c r="D92" s="15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="93" spans="2:4" x14ac:dyDescent="0.25">
@@ -1338,7 +1314,7 @@
         <v>305</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D93" s="5" t="s">
         <v>48</v>
@@ -1363,7 +1339,7 @@
         <v>3250</v>
       </c>
       <c r="D95" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="96" spans="2:4" x14ac:dyDescent="0.25">
@@ -1371,13 +1347,13 @@
         <v>308</v>
       </c>
       <c r="C96" s="9">
-        <v>2305</v>
+        <v>2309</v>
       </c>
       <c r="D96" s="9" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="97" spans="2:4" x14ac:dyDescent="0.25">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="97" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B97" s="2">
         <v>309</v>
       </c>
@@ -1388,7 +1364,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="98" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B98" s="2" t="s">
         <v>31</v>
       </c>
@@ -1396,10 +1372,13 @@
         <v>1101</v>
       </c>
       <c r="D98" s="21" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="99" spans="2:4" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+      <c r="E98" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="99" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B99" s="2" t="s">
         <v>32</v>
       </c>
@@ -1407,10 +1386,10 @@
         <v>8322</v>
       </c>
       <c r="D99" s="24" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="100" spans="2:4" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="100" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B100" s="2" t="s">
         <v>33</v>
       </c>
@@ -1418,10 +1397,10 @@
         <v>1300</v>
       </c>
       <c r="D100" s="26" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="101" spans="2:4" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="101" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B101" s="2" t="s">
         <v>34</v>
       </c>
@@ -1429,10 +1408,10 @@
         <v>3255</v>
       </c>
       <c r="D101" s="26" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="102" spans="2:4" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="102" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B102" s="2" t="s">
         <v>35</v>
       </c>
@@ -1440,10 +1419,10 @@
         <v>3252</v>
       </c>
       <c r="D102" s="26" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="103" spans="2:4" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="103" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B103" s="2" t="s">
         <v>36</v>
       </c>
@@ -1451,10 +1430,10 @@
         <v>2310</v>
       </c>
       <c r="D103" s="26" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="104" spans="2:4" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="104" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B104" s="2">
         <v>310</v>
       </c>
@@ -1462,10 +1441,10 @@
         <v>26</v>
       </c>
       <c r="D104" s="26" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="105" spans="2:4" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="105" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B105" s="2">
         <v>311</v>
       </c>
@@ -1473,10 +1452,10 @@
         <v>4000</v>
       </c>
       <c r="D105" s="28" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="106" spans="2:4" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="106" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B106" s="2">
         <v>312</v>
       </c>
@@ -1484,10 +1463,10 @@
         <v>3251</v>
       </c>
       <c r="D106" s="28" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="107" spans="2:4" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="107" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B107" s="1">
         <v>313</v>
       </c>
@@ -1495,10 +1474,10 @@
         <v>2254</v>
       </c>
       <c r="D107" s="11" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="108" spans="2:4" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="108" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B108" s="2">
         <v>314</v>
       </c>
@@ -1506,10 +1485,10 @@
         <v>1255</v>
       </c>
       <c r="D108" s="37" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="109" spans="2:4" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="109" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B109" s="1">
         <v>315</v>
       </c>
@@ -1517,10 +1496,10 @@
         <v>3256</v>
       </c>
       <c r="D109" s="37" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="110" spans="2:4" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="110" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B110" s="2">
         <v>316</v>
       </c>
@@ -1528,10 +1507,10 @@
         <v>2255</v>
       </c>
       <c r="D110" s="37" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="111" spans="2:4" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="111" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B111" s="1">
         <v>317</v>
       </c>
@@ -1542,7 +1521,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="112" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B112" s="2">
         <v>318</v>
       </c>
@@ -1550,7 +1529,7 @@
         <v>3251</v>
       </c>
       <c r="D112" s="40" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="113" spans="2:4" x14ac:dyDescent="0.25">
@@ -1561,7 +1540,7 @@
         <v>3253</v>
       </c>
       <c r="D113" s="28" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="114" spans="2:4" x14ac:dyDescent="0.25">
@@ -1572,7 +1551,7 @@
         <v>2320</v>
       </c>
       <c r="D114" s="28" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="115" spans="2:4" x14ac:dyDescent="0.25">
@@ -1594,7 +1573,7 @@
         <v>3251</v>
       </c>
       <c r="D116" s="54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="117" spans="2:4" x14ac:dyDescent="0.25">
@@ -1602,10 +1581,10 @@
         <v>40</v>
       </c>
       <c r="C117" s="55" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D117" s="54" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="118" spans="2:4" x14ac:dyDescent="0.25">
@@ -1625,7 +1604,7 @@
         <v>3254</v>
       </c>
       <c r="D119" s="54" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="120" spans="2:4" x14ac:dyDescent="0.25">
@@ -1636,7 +1615,7 @@
         <v>26</v>
       </c>
       <c r="D120" s="26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="121" spans="2:4" x14ac:dyDescent="0.25">
@@ -1647,7 +1626,7 @@
         <v>1309</v>
       </c>
       <c r="D121" s="51" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="122" spans="2:4" x14ac:dyDescent="0.25">
@@ -1658,7 +1637,7 @@
         <v>3252</v>
       </c>
       <c r="D122" s="49" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="123" spans="2:4" x14ac:dyDescent="0.25">
@@ -1669,7 +1648,7 @@
         <v>2200</v>
       </c>
       <c r="D123" s="46" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="124" spans="2:4" x14ac:dyDescent="0.25">
@@ -1702,7 +1681,7 @@
         <v>1300</v>
       </c>
       <c r="D126" s="26" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="127" spans="2:4" x14ac:dyDescent="0.25">
@@ -1713,7 +1692,7 @@
         <v>3255</v>
       </c>
       <c r="D127" s="26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="128" spans="2:4" x14ac:dyDescent="0.25">
@@ -1724,7 +1703,7 @@
         <v>3252</v>
       </c>
       <c r="D128" s="26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="129" spans="2:4" x14ac:dyDescent="0.25">
@@ -1735,7 +1714,7 @@
         <v>2326</v>
       </c>
       <c r="D129" s="26" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="130" spans="2:4" x14ac:dyDescent="0.25">
@@ -1746,28 +1725,28 @@
         <v>26</v>
       </c>
       <c r="D130" s="26" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="131" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B131" s="1">
         <v>327</v>
       </c>
-      <c r="C131" s="59">
+      <c r="C131" s="56">
         <v>2254</v>
       </c>
-      <c r="D131" s="60" t="s">
-        <v>65</v>
+      <c r="D131" s="57" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="132" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B132" s="1">
         <v>328</v>
       </c>
-      <c r="C132" s="62">
+      <c r="C132" s="59">
         <v>0</v>
       </c>
-      <c r="D132" s="63" t="s">
+      <c r="D132" s="60" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1775,48 +1754,46 @@
       <c r="B133" s="1">
         <v>329</v>
       </c>
-      <c r="C133" s="62">
+      <c r="C133" s="59">
         <v>7314</v>
       </c>
-      <c r="D133" s="64" t="s">
-        <v>83</v>
+      <c r="D133" s="61" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="134" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B134" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C134" s="56" t="s">
+        <v>78</v>
+      </c>
+      <c r="C134" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D134" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="D134" s="57" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="135" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B135" s="1"/>
-      <c r="C135" s="56"/>
-      <c r="D135" s="57"/>
+      <c r="C135" s="3"/>
+      <c r="D135" s="1"/>
     </row>
     <row r="136" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B136" s="1"/>
-      <c r="C136" s="56"/>
-      <c r="D136" s="57"/>
+      <c r="C136" s="3"/>
+      <c r="D136" s="1"/>
     </row>
     <row r="137" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B137" s="1"/>
-      <c r="C137" s="57"/>
-      <c r="D137" s="57"/>
+      <c r="C137" s="1"/>
+      <c r="D137" s="1"/>
     </row>
     <row r="138" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B138" s="1"/>
-      <c r="C138" s="57"/>
-      <c r="D138" s="57"/>
+      <c r="C138" s="1"/>
+      <c r="D138" s="1"/>
     </row>
     <row r="139" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B139" s="1"/>
-      <c r="C139" s="58"/>
-      <c r="D139" s="58"/>
     </row>
     <row r="140" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B140" s="1"/>

</xml_diff>